<commit_message>
additional ssx continuous source areas requested additions
</commit_message>
<xml_diff>
--- a/gis/xlsx/ECF-200-ZP1-25-0092/Table-A-2-Candidate-Wells/Table-A-2-Candidate-Wells.xlsx
+++ b/gis/xlsx/ECF-200-ZP1-25-0092/Table-A-2-Candidate-Wells/Table-A-2-Candidate-Wells.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\INTERA\hanford\CPCCO.M001.MRA-TOR-93\gis\xlsx\ECF-200-ZP1-25-0092\Table-A-2-Candidate-Wells\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C10A7FDC-9C9F-465C-9F8C-2C1BEB17D3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39296BE-990C-4E1A-A555-B2100295E617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B33F18B-1793-48BB-87B6-67DE977F3001}"/>
   </bookViews>
@@ -1099,7 +1099,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1108,8 +1108,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5196,38 +5194,38 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="4" t="s">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>92</v>
       </c>
-      <c r="B108" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C108" s="5">
+      <c r="B108" t="s">
+        <v>2</v>
+      </c>
+      <c r="C108" s="3">
         <v>566090.04599999997</v>
       </c>
-      <c r="D108" s="5">
+      <c r="D108" s="3">
         <v>135729.04500000001</v>
       </c>
-      <c r="E108" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F108" s="4" t="s">
+      <c r="E108" t="s">
+        <v>3</v>
+      </c>
+      <c r="F108" t="s">
         <v>9</v>
       </c>
-      <c r="G108" s="5">
+      <c r="G108" s="3">
         <v>213.137</v>
       </c>
-      <c r="H108" s="5">
+      <c r="H108" s="3">
         <v>137.91540800000001</v>
       </c>
-      <c r="I108" s="5">
+      <c r="I108" s="3">
         <v>130.289312</v>
       </c>
-      <c r="J108" s="5">
+      <c r="J108" s="3">
         <v>134.10236</v>
       </c>
-      <c r="K108" s="4" t="s">
+      <c r="K108" t="s">
         <v>5</v>
       </c>
     </row>
@@ -6207,38 +6205,38 @@
         <v>5</v>
       </c>
     </row>
-    <row r="137" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A137" s="4" t="s">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
         <v>123</v>
       </c>
-      <c r="B137" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C137" s="5">
+      <c r="B137" t="s">
+        <v>50</v>
+      </c>
+      <c r="C137" s="3">
         <v>567313.04</v>
       </c>
-      <c r="D137" s="5">
+      <c r="D137" s="3">
         <v>135547.01999999999</v>
       </c>
-      <c r="E137" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F137" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="G137" s="5">
+      <c r="E137" t="s">
+        <v>3</v>
+      </c>
+      <c r="F137" t="s">
+        <v>4</v>
+      </c>
+      <c r="G137" s="3">
         <v>214.261</v>
       </c>
-      <c r="H137" s="5">
+      <c r="H137" s="3">
         <v>125.957392</v>
       </c>
-      <c r="I137" s="5">
+      <c r="I137" s="3">
         <v>89.381391999999906</v>
       </c>
-      <c r="J137" s="5">
+      <c r="J137" s="3">
         <v>107.669392</v>
       </c>
-      <c r="K137" s="4" t="s">
+      <c r="K137" t="s">
         <v>27</v>
       </c>
     </row>
@@ -10994,38 +10992,38 @@
         <v>5</v>
       </c>
     </row>
-    <row r="274" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A274" s="4" t="s">
+    <row r="274" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
         <v>238</v>
       </c>
-      <c r="B274" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C274" s="4">
+      <c r="B274" t="s">
+        <v>50</v>
+      </c>
+      <c r="C274">
         <v>571219.09699999995</v>
       </c>
-      <c r="D274" s="4">
+      <c r="D274">
         <v>134997.28200000001</v>
       </c>
-      <c r="E274" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F274" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="G274" s="4">
+      <c r="E274" t="s">
+        <v>3</v>
+      </c>
+      <c r="F274" t="s">
+        <v>4</v>
+      </c>
+      <c r="G274">
         <v>227.261</v>
       </c>
-      <c r="H274" s="4">
+      <c r="H274">
         <v>125.427319999999</v>
       </c>
-      <c r="I274" s="4">
+      <c r="I274">
         <v>119.331319999999</v>
       </c>
-      <c r="J274" s="4">
+      <c r="J274">
         <v>122.379319999999</v>
       </c>
-      <c r="K274" s="4" t="s">
+      <c r="K274" t="s">
         <v>5</v>
       </c>
     </row>
@@ -11204,38 +11202,38 @@
         <v>5</v>
       </c>
     </row>
-    <row r="280" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A280" s="4" t="s">
+    <row r="280" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
         <v>242</v>
       </c>
-      <c r="B280" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C280" s="4">
+      <c r="B280" t="s">
+        <v>50</v>
+      </c>
+      <c r="C280">
         <v>569084.11</v>
       </c>
-      <c r="D280" s="4">
+      <c r="D280">
         <v>135325.57999999999</v>
       </c>
-      <c r="E280" s="4" t="s">
+      <c r="E280" t="s">
         <v>7</v>
       </c>
-      <c r="F280" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="G280" s="4">
+      <c r="F280" t="s">
+        <v>4</v>
+      </c>
+      <c r="G280">
         <v>225.93299999999999</v>
       </c>
-      <c r="H280" s="4">
+      <c r="H280">
         <v>105.329735999999</v>
       </c>
-      <c r="I280" s="4">
+      <c r="I280">
         <v>100.75163999999999</v>
       </c>
-      <c r="J280" s="4">
+      <c r="J280">
         <v>103.040688</v>
       </c>
-      <c r="K280" s="4" t="s">
+      <c r="K280" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>